<commit_message>
update for refresh dashboard
</commit_message>
<xml_diff>
--- a/Real Estate Analysis/Real_Estate_Dashboard_Template.xlsx
+++ b/Real Estate Analysis/Real_Estate_Dashboard_Template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f1bc5d2f802a0ef/Documents/edu2019/python/Projects/real-estate-revenue-analytics/Real Estate Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="11_5D765F0B13A2E543BDD38B6207B5A4637B504471" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FF7A255-7028-4A5D-91D5-633887B67A8B}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="11_5D765F0B13A2E543BDD38B6207B5A4637B504471" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDD3CC4F-97E6-44FD-9ACE-941EF0E61C91}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1620" yWindow="336" windowWidth="21600" windowHeight="10200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -344,7 +344,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -429,13 +429,13 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -449,116 +449,6 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1789,6 +1679,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2074,6 +1968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -2149,6 +2044,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C4418E7-B22B-4AEF-BC09-70F06BE54830}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2812,6 +2708,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5174A03-8012-4B99-ACDD-0C1EBBE74084}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2942,11 +2839,11 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G5">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Above Market"</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Below Market"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"Above Market"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2956,6 +2853,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFF2FF3-A0E7-4FE5-9D3C-3F3869097C7B}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -3714,6 +3612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B302EE0A-3E93-4FF1-919A-03D61F6EC839}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:D74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -4760,6 +4659,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr codeName="Sheet6"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>